<commit_message>
Validation faite pour toutes les PWM
</commit_message>
<xml_diff>
--- a/src/1_FMK/FMK_HAL/FMK_IO/Doc/Validation_FMKIO.xlsx
+++ b/src/1_FMK/FMK_HAL/FMK_IO/Doc/Validation_FMKIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_designHRTIM\src\1_FMK\FMK_HAL\FMK_IO\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391B05E6-5B02-4AF9-AB7D-2F028AE5AEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC392AE0-327D-47F5-9C98-E9A968896EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B654A100-FC4B-4AD6-8CD5-7BE8F9D1ACE1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="95">
   <si>
     <t>Signal Name</t>
   </si>
@@ -150,16 +150,193 @@
   </si>
   <si>
     <t>TimeDiff 3 %</t>
+  </si>
+  <si>
+    <t>Commit</t>
+  </si>
+  <si>
+    <t>PWM_7</t>
+  </si>
+  <si>
+    <t>PC2</t>
+  </si>
+  <si>
+    <t>ADV</t>
+  </si>
+  <si>
+    <t>PWM_6</t>
+  </si>
+  <si>
+    <t>PB2</t>
+  </si>
+  <si>
+    <t>PWM_5</t>
+  </si>
+  <si>
+    <t>PC7</t>
+  </si>
+  <si>
+    <t>PWM_4</t>
+  </si>
+  <si>
+    <t>PB15</t>
+  </si>
+  <si>
+    <t>BSC</t>
+  </si>
+  <si>
+    <t>PWM_3</t>
+  </si>
+  <si>
+    <t>PWM_2</t>
+  </si>
+  <si>
+    <t>PWM_1</t>
+  </si>
+  <si>
+    <t>PC12</t>
+  </si>
+  <si>
+    <t>PB9</t>
+  </si>
+  <si>
+    <t>PB4</t>
+  </si>
+  <si>
+    <t>de6e41b2</t>
+  </si>
+  <si>
+    <t>de6e41b3</t>
+  </si>
+  <si>
+    <t>de6e41b4</t>
+  </si>
+  <si>
+    <t>de6e41b5</t>
+  </si>
+  <si>
+    <t>de6e41b6</t>
+  </si>
+  <si>
+    <t>de6e41b7</t>
+  </si>
+  <si>
+    <t>de6e41b8</t>
+  </si>
+  <si>
+    <t>de6e41b9</t>
+  </si>
+  <si>
+    <t>de6e41b10</t>
+  </si>
+  <si>
+    <t>de6e41b11</t>
+  </si>
+  <si>
+    <t>de6e41b12</t>
+  </si>
+  <si>
+    <t>de6e41b13</t>
+  </si>
+  <si>
+    <t>de6e41b14</t>
+  </si>
+  <si>
+    <t>de6e41b15</t>
+  </si>
+  <si>
+    <t>de6e41b16</t>
+  </si>
+  <si>
+    <t>de6e41b17</t>
+  </si>
+  <si>
+    <t>de6e41b18</t>
+  </si>
+  <si>
+    <t>de6e41b19</t>
+  </si>
+  <si>
+    <t>de6e41b20</t>
+  </si>
+  <si>
+    <t>de6e41b21</t>
+  </si>
+  <si>
+    <t>de6e41b22</t>
+  </si>
+  <si>
+    <t>de6e41b23</t>
+  </si>
+  <si>
+    <t>de6e41b24</t>
+  </si>
+  <si>
+    <t>de6e41b25</t>
+  </si>
+  <si>
+    <t>de6e41b26</t>
+  </si>
+  <si>
+    <t>de6e41b27</t>
+  </si>
+  <si>
+    <t>de6e41b28</t>
+  </si>
+  <si>
+    <t>de6e41b29</t>
+  </si>
+  <si>
+    <t>de6e41b30</t>
+  </si>
+  <si>
+    <t>de6e41b31</t>
+  </si>
+  <si>
+    <t>de6e41b32</t>
+  </si>
+  <si>
+    <t>de6e41b33</t>
+  </si>
+  <si>
+    <t>de6e41b34</t>
+  </si>
+  <si>
+    <t>de6e41b35</t>
+  </si>
+  <si>
+    <t>de6e41b36</t>
+  </si>
+  <si>
+    <t>de6e41b37</t>
+  </si>
+  <si>
+    <t>de6e41b38</t>
+  </si>
+  <si>
+    <t>de6e41b39</t>
+  </si>
+  <si>
+    <t>de6e41b40</t>
+  </si>
+  <si>
+    <t>de6e41b41</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -212,9 +389,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D85C0DC8-4B53-4406-A1A5-399EBE39C1B4}" name="Tableau1" displayName="Tableau1" ref="D19:J40" totalsRowShown="0">
-  <autoFilter ref="D19:J40" xr:uid="{D85C0DC8-4B53-4406-A1A5-399EBE39C1B4}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D85C0DC8-4B53-4406-A1A5-399EBE39C1B4}" name="Tableau1" displayName="Tableau1" ref="D19:K61" totalsRowShown="0">
+  <autoFilter ref="D19:K61" xr:uid="{D85C0DC8-4B53-4406-A1A5-399EBE39C1B4}"/>
+  <tableColumns count="8">
     <tableColumn id="7" xr3:uid="{85E5D1C5-8EBA-4AC8-8A4B-D875ED539E63}" name="Signal Name"/>
     <tableColumn id="1" xr3:uid="{E9808153-524F-4B4B-B49A-8E4CBC854CC4}" name="Bsp Name"/>
     <tableColumn id="2" xr3:uid="{BFB92BD7-0E9B-4907-AB99-EC5156E336C5}" name="Timer Type"/>
@@ -222,6 +399,7 @@
     <tableColumn id="4" xr3:uid="{093DFA66-FA3A-4A96-8CEA-600972E0E848}" name="Etat "/>
     <tableColumn id="5" xr3:uid="{170D6092-1ABB-42BA-A6D4-CCAD771BA109}" name="Comment"/>
     <tableColumn id="6" xr3:uid="{E3CAC770-BD93-4EF8-8099-8BD1FF7E1471}" name="incertitude"/>
+    <tableColumn id="8" xr3:uid="{C4C46754-F9A3-4572-B423-FA173B0F0E83}" name="Commit"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -555,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{634BA75F-9645-4262-9D67-E06FEFBAB9A9}">
-  <dimension ref="B3:J40"/>
+  <dimension ref="B3:K61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27" customWidth="1"/>
@@ -617,7 +795,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="4:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D19" t="s">
         <v>0</v>
       </c>
@@ -639,8 +817,11 @@
       <c r="J19" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="20" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D20" t="s">
         <v>5</v>
       </c>
@@ -659,8 +840,11 @@
       <c r="J20" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="21" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D21" t="s">
         <v>5</v>
       </c>
@@ -676,8 +860,11 @@
       <c r="H21" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="22" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D22" t="s">
         <v>5</v>
       </c>
@@ -693,8 +880,11 @@
       <c r="H22" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="23" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D23" t="s">
         <v>21</v>
       </c>
@@ -710,8 +900,11 @@
       <c r="H23" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="24" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D24" t="s">
         <v>21</v>
       </c>
@@ -727,8 +920,11 @@
       <c r="H24" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="25" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D25" t="s">
         <v>22</v>
       </c>
@@ -744,8 +940,11 @@
       <c r="H25" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="26" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K25" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D26" t="s">
         <v>22</v>
       </c>
@@ -761,8 +960,11 @@
       <c r="H26" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="27" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K26" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D27" t="s">
         <v>24</v>
       </c>
@@ -778,8 +980,11 @@
       <c r="H27" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="28" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D28" t="s">
         <v>24</v>
       </c>
@@ -795,8 +1000,11 @@
       <c r="H28" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="29" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K28" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="29" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D29" t="s">
         <v>26</v>
       </c>
@@ -812,8 +1020,11 @@
       <c r="H29" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="30" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K29" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="30" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D30" t="s">
         <v>26</v>
       </c>
@@ -829,8 +1040,11 @@
       <c r="H30" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="31" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K30" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="31" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D31" t="s">
         <v>28</v>
       </c>
@@ -846,8 +1060,11 @@
       <c r="H31" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="32" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K31" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D32" t="s">
         <v>28</v>
       </c>
@@ -863,8 +1080,11 @@
       <c r="H32" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="33" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K32" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D33" t="s">
         <v>22</v>
       </c>
@@ -883,8 +1103,11 @@
       <c r="J33" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="34" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K33" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="34" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D34" t="s">
         <v>22</v>
       </c>
@@ -900,8 +1123,11 @@
       <c r="H34" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="35" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K34" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D35" t="s">
         <v>21</v>
       </c>
@@ -917,8 +1143,11 @@
       <c r="H35" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="36" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K35" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D36" t="s">
         <v>21</v>
       </c>
@@ -934,8 +1163,11 @@
       <c r="H36" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="37" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K36" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D37" t="s">
         <v>5</v>
       </c>
@@ -951,8 +1183,11 @@
       <c r="H37" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="38" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K37" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D38" t="s">
         <v>34</v>
       </c>
@@ -968,8 +1203,11 @@
       <c r="H38" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="39" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K38" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D39" t="s">
         <v>35</v>
       </c>
@@ -985,8 +1223,11 @@
       <c r="H39" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="40" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="K39" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="40" spans="4:11" x14ac:dyDescent="0.3">
       <c r="D40" t="s">
         <v>36</v>
       </c>
@@ -1002,8 +1243,432 @@
       <c r="H40" t="s">
         <v>13</v>
       </c>
+      <c r="K40" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="41" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D41" t="s">
+        <v>39</v>
+      </c>
+      <c r="E41" t="s">
+        <v>40</v>
+      </c>
+      <c r="F41" t="s">
+        <v>41</v>
+      </c>
+      <c r="G41" t="s">
+        <v>9</v>
+      </c>
+      <c r="H41" t="s">
+        <v>13</v>
+      </c>
+      <c r="K41" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="42" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D42" t="s">
+        <v>39</v>
+      </c>
+      <c r="E42" t="s">
+        <v>40</v>
+      </c>
+      <c r="F42" t="s">
+        <v>41</v>
+      </c>
+      <c r="G42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" t="s">
+        <v>13</v>
+      </c>
+      <c r="K42" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="43" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D43" t="s">
+        <v>39</v>
+      </c>
+      <c r="E43" t="s">
+        <v>40</v>
+      </c>
+      <c r="F43" t="s">
+        <v>41</v>
+      </c>
+      <c r="G43" t="s">
+        <v>19</v>
+      </c>
+      <c r="H43" t="s">
+        <v>13</v>
+      </c>
+      <c r="K43" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="44" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D44" t="s">
+        <v>39</v>
+      </c>
+      <c r="E44" t="s">
+        <v>40</v>
+      </c>
+      <c r="F44" t="s">
+        <v>41</v>
+      </c>
+      <c r="G44" t="s">
+        <v>30</v>
+      </c>
+      <c r="H44" t="s">
+        <v>13</v>
+      </c>
+      <c r="K44" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D45" t="s">
+        <v>39</v>
+      </c>
+      <c r="E45" t="s">
+        <v>40</v>
+      </c>
+      <c r="F45" t="s">
+        <v>41</v>
+      </c>
+      <c r="G45" t="s">
+        <v>32</v>
+      </c>
+      <c r="H45" t="s">
+        <v>13</v>
+      </c>
+      <c r="K45" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="46" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D46" t="s">
+        <v>42</v>
+      </c>
+      <c r="E46" t="s">
+        <v>43</v>
+      </c>
+      <c r="F46" t="s">
+        <v>41</v>
+      </c>
+      <c r="G46" t="s">
+        <v>9</v>
+      </c>
+      <c r="H46" t="s">
+        <v>13</v>
+      </c>
+      <c r="K46" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="47" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D47" t="s">
+        <v>42</v>
+      </c>
+      <c r="E47" t="s">
+        <v>43</v>
+      </c>
+      <c r="F47" t="s">
+        <v>41</v>
+      </c>
+      <c r="G47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" t="s">
+        <v>13</v>
+      </c>
+      <c r="K47" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="48" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D48" t="s">
+        <v>42</v>
+      </c>
+      <c r="E48" t="s">
+        <v>43</v>
+      </c>
+      <c r="F48" t="s">
+        <v>41</v>
+      </c>
+      <c r="G48" t="s">
+        <v>30</v>
+      </c>
+      <c r="H48" t="s">
+        <v>13</v>
+      </c>
+      <c r="K48" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="49" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D49" t="s">
+        <v>42</v>
+      </c>
+      <c r="E49" t="s">
+        <v>43</v>
+      </c>
+      <c r="F49" t="s">
+        <v>41</v>
+      </c>
+      <c r="G49" t="s">
+        <v>32</v>
+      </c>
+      <c r="H49" t="s">
+        <v>13</v>
+      </c>
+      <c r="K49" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="50" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D50" t="s">
+        <v>44</v>
+      </c>
+      <c r="E50" t="s">
+        <v>45</v>
+      </c>
+      <c r="F50" t="s">
+        <v>41</v>
+      </c>
+      <c r="G50" t="s">
+        <v>9</v>
+      </c>
+      <c r="H50" t="s">
+        <v>13</v>
+      </c>
+      <c r="K50" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="51" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D51" t="s">
+        <v>44</v>
+      </c>
+      <c r="E51" t="s">
+        <v>45</v>
+      </c>
+      <c r="F51" t="s">
+        <v>41</v>
+      </c>
+      <c r="G51" t="s">
+        <v>15</v>
+      </c>
+      <c r="H51" t="s">
+        <v>13</v>
+      </c>
+      <c r="K51" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="52" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D52" t="s">
+        <v>44</v>
+      </c>
+      <c r="E52" t="s">
+        <v>45</v>
+      </c>
+      <c r="F52" t="s">
+        <v>48</v>
+      </c>
+      <c r="G52" t="s">
+        <v>30</v>
+      </c>
+      <c r="H52" t="s">
+        <v>13</v>
+      </c>
+      <c r="K52" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="53" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D53" t="s">
+        <v>44</v>
+      </c>
+      <c r="E53" t="s">
+        <v>45</v>
+      </c>
+      <c r="F53" t="s">
+        <v>48</v>
+      </c>
+      <c r="G53" t="s">
+        <v>32</v>
+      </c>
+      <c r="H53" t="s">
+        <v>13</v>
+      </c>
+      <c r="K53" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="54" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D54" t="s">
+        <v>46</v>
+      </c>
+      <c r="E54" t="s">
+        <v>47</v>
+      </c>
+      <c r="F54" t="s">
+        <v>48</v>
+      </c>
+      <c r="G54" t="s">
+        <v>9</v>
+      </c>
+      <c r="H54" t="s">
+        <v>13</v>
+      </c>
+      <c r="K54" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="55" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D55" t="s">
+        <v>46</v>
+      </c>
+      <c r="E55" t="s">
+        <v>47</v>
+      </c>
+      <c r="F55" t="s">
+        <v>48</v>
+      </c>
+      <c r="G55" t="s">
+        <v>15</v>
+      </c>
+      <c r="H55" t="s">
+        <v>13</v>
+      </c>
+      <c r="K55" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="56" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D56" t="s">
+        <v>49</v>
+      </c>
+      <c r="E56" t="s">
+        <v>52</v>
+      </c>
+      <c r="F56" t="s">
+        <v>48</v>
+      </c>
+      <c r="G56" t="s">
+        <v>9</v>
+      </c>
+      <c r="H56" t="s">
+        <v>13</v>
+      </c>
+      <c r="K56" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="57" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D57" t="s">
+        <v>49</v>
+      </c>
+      <c r="E57" t="s">
+        <v>52</v>
+      </c>
+      <c r="F57" t="s">
+        <v>48</v>
+      </c>
+      <c r="G57" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" t="s">
+        <v>13</v>
+      </c>
+      <c r="K57" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="58" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D58" t="s">
+        <v>50</v>
+      </c>
+      <c r="E58" t="s">
+        <v>53</v>
+      </c>
+      <c r="F58" t="s">
+        <v>48</v>
+      </c>
+      <c r="G58" t="s">
+        <v>9</v>
+      </c>
+      <c r="H58" t="s">
+        <v>13</v>
+      </c>
+      <c r="K58" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="59" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D59" t="s">
+        <v>50</v>
+      </c>
+      <c r="E59" t="s">
+        <v>53</v>
+      </c>
+      <c r="F59" t="s">
+        <v>48</v>
+      </c>
+      <c r="G59" t="s">
+        <v>15</v>
+      </c>
+      <c r="H59" t="s">
+        <v>13</v>
+      </c>
+      <c r="K59" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="60" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D60" t="s">
+        <v>51</v>
+      </c>
+      <c r="E60" t="s">
+        <v>54</v>
+      </c>
+      <c r="F60" t="s">
+        <v>48</v>
+      </c>
+      <c r="G60" t="s">
+        <v>9</v>
+      </c>
+      <c r="H60" t="s">
+        <v>13</v>
+      </c>
+      <c r="K60" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="61" spans="4:11" x14ac:dyDescent="0.3">
+      <c r="D61" t="s">
+        <v>51</v>
+      </c>
+      <c r="E61" t="s">
+        <v>54</v>
+      </c>
+      <c r="F61" t="s">
+        <v>48</v>
+      </c>
+      <c r="G61" t="s">
+        <v>15</v>
+      </c>
+      <c r="H61" t="s">
+        <v>13</v>
+      </c>
+      <c r="K61" t="s">
+        <v>94</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
     <tablePart r:id="rId1"/>

</xml_diff>